<commit_message>
Update brief title to FSO Briefing heading
https://claude.ai/code/session_01UdifTpwTrGAc4BWznJJNRd
</commit_message>
<xml_diff>
--- a/travel_brief/Foreign_Travel_Brief_Thailand.xlsx
+++ b/travel_brief/Foreign_Travel_Brief_Thailand.xlsx
@@ -491,14 +491,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>International Foreign Travel Brief</t>
+          <t>Cleared &amp; Non-Cleared Foreign Travel Reporting — Facility Security Officer (FSO) Briefing</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cleared &amp; Non-Cleared Foreign Travel Reporting — Facility Security Officer (FSO)</t>
+          <t>International Foreign Travel Brief</t>
         </is>
       </c>
     </row>

</xml_diff>